<commit_message>
login added to batch
</commit_message>
<xml_diff>
--- a/batch_search_test_input.xlsx
+++ b/batch_search_test_input.xlsx
@@ -609,7 +609,7 @@
       </c>
       <c r="K2" t="inlineStr">
         <is>
-          <t>02 Jun 2026</t>
+          <t>06 Jun 2026</t>
         </is>
       </c>
       <c r="L2" t="inlineStr">
@@ -703,7 +703,7 @@
       </c>
       <c r="K3" t="inlineStr">
         <is>
-          <t>02 Jun 2026</t>
+          <t>06 Jun 2026</t>
         </is>
       </c>
       <c r="L3" t="inlineStr">

</xml_diff>